<commit_message>
Correct AEON RYS documentation accuracy notes
</commit_message>
<xml_diff>
--- a/docs/qwen36-aeon-rys-15-20/assets/qwen36_aeon_rys_stats.xlsx
+++ b/docs/qwen36-aeon-rys-15-20/assets/qwen36_aeon_rys_stats.xlsx
@@ -1962,7 +1962,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -1972,7 +1972,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>